<commit_message>
Update EDA notebook and README with final risk scores, maps, and insights
</commit_message>
<xml_diff>
--- a/data/earthquake_zones_by_county.xlsx
+++ b/data/earthquake_zones_by_county.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/annapiterskaya/Desktop/earthquake-insurance-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40741786-F7D6-4F4C-9FD4-6769042F0400}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{641C1982-88A8-7543-ACE4-B921AE56EE70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20720" xr2:uid="{C5914727-A51A-7D45-BF56-4B0DDA0A7542}"/>
+    <workbookView xWindow="40" yWindow="740" windowWidth="35840" windowHeight="20720" xr2:uid="{C5914727-A51A-7D45-BF56-4B0DDA0A7542}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -74,9 +74,6 @@
     <t>Yolo</t>
   </si>
   <si>
-    <t>Tuolomne</t>
-  </si>
-  <si>
     <t>Sutter</t>
   </si>
   <si>
@@ -218,9 +215,6 @@
     <t>Lake</t>
   </si>
   <si>
-    <t>Humbolt</t>
-  </si>
-  <si>
     <t>Del Norte</t>
   </si>
   <si>
@@ -240,13 +234,19 @@
   </si>
   <si>
     <t>county</t>
+  </si>
+  <si>
+    <t>Tuolumne</t>
+  </si>
+  <si>
+    <t>Humboldt</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -260,6 +260,12 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -282,9 +288,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -619,304 +626,305 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0598184E-8EAA-7F41-AA81-A31DEF9431E8}">
-  <dimension ref="A1:B59"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>61</v>
-      </c>
-      <c r="B6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>60</v>
-      </c>
       <c r="B7" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B8" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B9" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B10" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B11" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B13" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B14" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B22" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B27" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B28" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B32" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B33" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B34" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B35" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B36" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B37" t="s">
         <v>9</v>
@@ -924,7 +932,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B38" t="s">
         <v>9</v>
@@ -932,7 +940,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B39" t="s">
         <v>9</v>
@@ -940,7 +948,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B40" t="s">
         <v>9</v>
@@ -948,7 +956,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B41" t="s">
         <v>9</v>
@@ -956,7 +964,7 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B42" t="s">
         <v>9</v>
@@ -964,7 +972,7 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B43" t="s">
         <v>9</v>
@@ -972,7 +980,7 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B44" t="s">
         <v>9</v>
@@ -980,7 +988,7 @@
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B45" t="s">
         <v>9</v>
@@ -988,7 +996,7 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B46" t="s">
         <v>9</v>
@@ -996,7 +1004,7 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B47" t="s">
         <v>9</v>
@@ -1004,7 +1012,7 @@
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B48" t="s">
         <v>9</v>
@@ -1012,7 +1020,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>12</v>
+        <v>66</v>
       </c>
       <c r="B49" t="s">
         <v>9</v>

</xml_diff>